<commit_message>
Expand verified journal profiles
</commit_message>
<xml_diff>
--- a/deliverables/AI4Polymer_journal_guide.xlsx
+++ b/deliverables/AI4Polymer_journal_guide.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rbfebe4d3fe404df1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal Database" sheetId="2" r:id="Recc26d93c763467c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Profiles" sheetId="3" r:id="R94b4d242445a4108"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Method" sheetId="4" r:id="R4ee740a9d2d04e81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rb4e33389e6f242e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal Database" sheetId="2" r:id="R10262395e8224392"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Profiles" sheetId="3" r:id="Rf0520ab3c8714dd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Method" sheetId="4" r:id="R3bd46666ef9a4a01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +66,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -98,6 +98,21 @@
         <x:fgColor rgb="FFFFF7F1"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF155E75"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF155E75"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF155E75"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -111,7 +126,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -171,6 +186,12 @@
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -212,7 +233,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PriorityProfiles" displayName="PriorityProfiles" ref="A1:N5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PriorityProfiles" displayName="PriorityProfiles" ref="A1:N12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Journal"/>
     <x:tableColumn id="2" name="WoS records"/>
@@ -515,7 +536,7 @@
         <x:v>Priority profiles with official detail</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D7" s="11"/>
       <x:c r="E7" s="11"/>
@@ -746,13 +767,13 @@
         <x:v>JIF 5.8（2025）；官网列 JCR Polymer Science Q1、CiteScore 分区 Q1（须按年份核对）。</x:v>
       </x:c>
       <x:c r="I2" s="25" t="str">
-        <x:v>投稿至首个编辑决定：13.4 天</x:v>
+        <x:v>投稿至首个编辑决定：13.4 天；接收到发表：2.7 天。官网称为 2026 上半年发表论文的中位数；不是首轮外审时长或投稿至接收。</x:v>
       </x:c>
       <x:c r="J2" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>投稿至接收</x:v>
       </x:c>
       <x:c r="K2" s="25" t="str">
-        <x:v>中位 2.7 天（接收到发表；2026H1）</x:v>
+        <x:v>未公开/待核验</x:v>
       </x:c>
       <x:c r="L2" s="25" t="str">
         <x:v>全 OA；APC CHF 2,700，适用税费另计；接受后开票。官网列机构 IOAP 与学会折扣。</x:v>
@@ -890,34 +911,34 @@
         <x:v>聚合物/高分子</x:v>
       </x:c>
       <x:c r="E4" s="25" t="str">
-        <x:v>根据期刊名称/学科线索的初步分类；需结合官网 aims &amp; scope 和近年相关文章判断。</x:v>
+        <x:v>基础聚合物科学定位强，涵盖合成、结构、物理化学、表征、加工及理论/模拟。聚合物信息学投稿应提出对高分子科学有解释力的发现，不宜只展示模型分数。</x:v>
       </x:c>
       <x:c r="F4" s="25" t="str">
-        <x:v>待核验：需查官网 Aims &amp; Scope</x:v>
+        <x:v>ACS 将其定位为发表前沿聚合物科学研究的同行评审期刊；理论、实验、模拟与跨学科工作均可考虑。</x:v>
       </x:c>
       <x:c r="G4" s="25" t="str">
-        <x:v>待核验：需查官网作者指南</x:v>
+        <x:v>Articles；期刊也刊发综述、观点/专题等类型，当前投稿分类与邀请要求以 ACS 作者指南为准。</x:v>
       </x:c>
       <x:c r="H4" s="25" t="str">
-        <x:v>未核验</x:v>
+        <x:v>JIF 5.7；5-year JIF 5.5；CiteScore 8.8（ACS Journal Metrics 页面，2026-06-17 数据快照；指标年份仍应按投稿时核对）。</x:v>
       </x:c>
       <x:c r="I4" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>ACS 中位数：投稿至无外审编辑决定 3.9 天；投稿至含同行评审决定 34 天；投稿至接收 86 天（含作者返修时间）；接收至 ASAP 8.4 天（含校样批准）。这些阶段不是单纯外审用时。</x:v>
       </x:c>
       <x:c r="J4" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>投稿至接收 86 天（含作者返修时间）</x:v>
       </x:c>
       <x:c r="K4" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>接收至 ASAP 8.4 天（含校样批准）</x:v>
       </x:c>
       <x:c r="L4" s="25" t="str">
-        <x:v>待核验</x:v>
+        <x:v>混合/可选 OA；可走订阅发表。OA APC 金额随 ACS 价目、币种、税费与机构协议变化，本次未核定应付总额。</x:v>
       </x:c>
       <x:c r="M4" s="25" t="str">
-        <x:v>未核验</x:v>
+        <x:v>American Chemical Society</x:v>
       </x:c>
       <x:c r="N4" s="25" t="str">
-        <x:v>待核验</x:v>
+        <x:v>0024-9297 (print); 1520-5835 (online)</x:v>
       </x:c>
       <x:c r="O4" s="25" t="str">
         <x:v>未公开/未找到可比官方统计</x:v>
@@ -944,10 +965,12 @@
         <x:v>待逐刊核验</x:v>
       </x:c>
       <x:c r="W4" s="25" t="str">
-        <x:v>基础目录（逐刊待核验）</x:v>
+        <x:v>官方资料已核验（重点期刊）</x:v>
       </x:c>
       <x:c r="X4" s="25" t="str">
-        <x:v>待核验：期刊官网</x:v>
+        <x:v>https://pubs.acs.org/journal/macromolecules
+https://pubs.acs.org/journal-metrics
+https://pubs.acs.org/mamobx/pages/info-for-authors</x:v>
       </x:c>
       <x:c r="Y4" s="25" t="str">
         <x:v>所给 WoS 汇总表频次；原检索期和窗口未提供</x:v>
@@ -1198,34 +1221,34 @@
         <x:v>工程/应用</x:v>
       </x:c>
       <x:c r="E8" s="25" t="str">
-        <x:v>根据期刊名称/学科线索的初步分类；需结合官网 aims &amp; scope 和近年相关文章判断。</x:v>
+        <x:v>适合将聚合物信息学与化工过程、反应/分离、能源/环境技术、规模化加工或可量化工程性能联系起来的研究。仅有材料性质预测、缺少化工问题或验证时匹配度较低。</x:v>
       </x:c>
       <x:c r="F8" s="25" t="str">
-        <x:v>待核验：需查官网 Aims &amp; Scope</x:v>
+        <x:v>工程应用驱动的化学工程研究；聚合物工作需清晰体现过程、系统或应用层面的化工价值。</x:v>
       </x:c>
       <x:c r="G8" s="25" t="str">
-        <x:v>待核验：需查官网作者指南</x:v>
+        <x:v>Research Articles、Review Articles、Short Communications 等；具体栏目和字数按最新版 Elsevier Guide for Authors 核验。</x:v>
       </x:c>
       <x:c r="H8" s="25" t="str">
-        <x:v>未核验</x:v>
+        <x:v>ScienceDirect 期刊页显示 Impact Factor 12.5、CiteScore 19.6（页面动态指标快照；年份口径应投稿前复核）。</x:v>
       </x:c>
       <x:c r="I8" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>官方公开页面未核到可比的投稿至首决、送外审首决、投稿至接收或接收到在线发表中位数；分别标记未公开。</x:v>
       </x:c>
       <x:c r="J8" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>投稿至接收或接收到在线发表中位数</x:v>
       </x:c>
       <x:c r="K8" s="25" t="str">
         <x:v>未公开/待核验</x:v>
       </x:c>
       <x:c r="L8" s="25" t="str">
-        <x:v>待核验</x:v>
+        <x:v>ScienceDirect 标注支持 OA；为订阅/混合路线的选择情况及最新 APC、税费和机构协议，本次未确认具体金额，投稿时查看官方 OA 成本计算器。</x:v>
       </x:c>
       <x:c r="M8" s="25" t="str">
-        <x:v>未核验</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="N8" s="25" t="str">
-        <x:v>待核验</x:v>
+        <x:v>1385-8947 (print); 1873-3212 (online)</x:v>
       </x:c>
       <x:c r="O8" s="25" t="str">
         <x:v>未公开/未找到可比官方统计</x:v>
@@ -1252,10 +1275,12 @@
         <x:v>待逐刊核验</x:v>
       </x:c>
       <x:c r="W8" s="25" t="str">
-        <x:v>基础目录（逐刊待核验）</x:v>
+        <x:v>官方资料已核验（重点期刊）</x:v>
       </x:c>
       <x:c r="X8" s="25" t="str">
-        <x:v>待核验：期刊官网</x:v>
+        <x:v>https://www.sciencedirect.com/journal/chemical-engineering-journal
+https://www.sciencedirect.com/journal/chemical-engineering-journal/publish/guide-for-authors
+https://www.sciencedirect.com/journal/chemical-engineering-journal/vol/226/suppl/C</x:v>
       </x:c>
       <x:c r="Y8" s="25" t="str">
         <x:v>所给 WoS 汇总表频次；原检索期和窗口未提供</x:v>
@@ -1287,13 +1312,13 @@
         <x:v>JIF 6.4、5 年 IF 6.9、CiteScore 8.8（ACS 页面，数据 as of 2025）。</x:v>
       </x:c>
       <x:c r="I9" s="25" t="str">
-        <x:v>首个同行评审决定中位数 31.3 天</x:v>
+        <x:v>首个同行评审决定中位数 31.3 天；投稿到接收 76.3 天；接收至 ASAP 9.6 天（ACS 页面，2025；口径并非每个处理阶段）。</x:v>
       </x:c>
       <x:c r="J9" s="25" t="str">
-        <x:v>中位 76.3 天（投稿至接收）</x:v>
+        <x:v>未公开/待核验</x:v>
       </x:c>
       <x:c r="K9" s="25" t="str">
-        <x:v>中位 9.6 天（接收至 ASAP；2025）</x:v>
+        <x:v>接收至 ASAP 9.6 天（ACS 页面，2025</x:v>
       </x:c>
       <x:c r="L9" s="25" t="str">
         <x:v>混合 OA，可选 CC BY/CC BY-NC-ND；非 OA 订阅路线可用。费用按 ACS 最新价目/协议核实。</x:v>
@@ -1431,34 +1456,34 @@
         <x:v>聚合物/高分子</x:v>
       </x:c>
       <x:c r="E11" s="25" t="str">
-        <x:v>根据期刊名称/学科线索的初步分类；需结合官网 aims &amp; scope 和近年相关文章判断。</x:v>
+        <x:v>传统聚合物科学与技术综合刊。匹配合成、结构/性能、物理化学、表征、加工、应用，以及具有明确高分子科学贡献的建模与机器学习研究。</x:v>
       </x:c>
       <x:c r="F11" s="25" t="str">
-        <x:v>待核验：需查官网 Aims &amp; Scope</x:v>
+        <x:v>覆盖聚合物科学和技术；计算研究应给出与聚合物现象、机制或应用相关的可验证贡献。</x:v>
       </x:c>
       <x:c r="G11" s="25" t="str">
-        <x:v>待核验：需查官网作者指南</x:v>
+        <x:v>Research/Regular Articles、Review Articles、Short Communications（以当前作者指南为准）。</x:v>
       </x:c>
       <x:c r="H11" s="25" t="str">
-        <x:v>未核验</x:v>
+        <x:v>ScienceDirect 官方期刊页面快照显示 Impact Factor 4.5、CiteScore 7.4；该快照指标年份未明确，不能作为当前年份保证值。</x:v>
       </x:c>
       <x:c r="I11" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>未核到官网公布的首个编辑决定、外审首决、投稿至接收和接收至在线发表中位数。</x:v>
       </x:c>
       <x:c r="J11" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>投稿至接收和接收至在线发表中位数</x:v>
       </x:c>
       <x:c r="K11" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>接收至在线发表中位数</x:v>
       </x:c>
       <x:c r="L11" s="25" t="str">
-        <x:v>待核验</x:v>
+        <x:v>ScienceDirect 标注支持 Open Access；按订阅/混合期刊路线处理。当前 APC、税费、协议覆盖需从官方作者端重新确认。</x:v>
       </x:c>
       <x:c r="M11" s="25" t="str">
-        <x:v>未核验</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="N11" s="25" t="str">
-        <x:v>待核验</x:v>
+        <x:v>0032-3861 (print); 1873-2291 (online)</x:v>
       </x:c>
       <x:c r="O11" s="25" t="str">
         <x:v>未公开/未找到可比官方统计</x:v>
@@ -1485,10 +1510,12 @@
         <x:v>待逐刊核验</x:v>
       </x:c>
       <x:c r="W11" s="25" t="str">
-        <x:v>基础目录（逐刊待核验）</x:v>
+        <x:v>官方资料已核验（重点期刊）</x:v>
       </x:c>
       <x:c r="X11" s="25" t="str">
-        <x:v>待核验：期刊官网</x:v>
+        <x:v>https://www.sciencedirect.com/journal/polymer
+https://www.sciencedirect.com/journal/polymer/publish/guide-for-authors
+https://www.sciencedirect.com/journal/polymer/vol/298/suppl/C</x:v>
       </x:c>
       <x:c r="Y11" s="25" t="str">
         <x:v>所给 WoS 汇总表频次；原检索期和窗口未提供</x:v>
@@ -1597,10 +1624,10 @@
         <x:v>JIF 13.1、5 年 JIF 13.7、SJR 2.943（2025）。</x:v>
       </x:c>
       <x:c r="I13" s="25" t="str">
-        <x:v>投稿至首个编辑决定中位数 14 天</x:v>
+        <x:v>投稿至首个编辑决定中位数 14 天；投稿至接收中位数 136 天（Springer Nature 官方，2025）。首决可能含编辑筛选。</x:v>
       </x:c>
       <x:c r="J13" s="25" t="str">
-        <x:v>中位 136 天（官方口径；不等于首轮外审）</x:v>
+        <x:v>投稿至接收中位数 136 天（Springer Nature 官方，2025）</x:v>
       </x:c>
       <x:c r="K13" s="25" t="str">
         <x:v>未公开/待核验</x:v>
@@ -1742,34 +1769,34 @@
         <x:v>计算/AI</x:v>
       </x:c>
       <x:c r="E15" s="25" t="str">
-        <x:v>根据期刊名称/学科线索的初步分类；需结合官网 aims &amp; scope 和近年相关文章判断。</x:v>
+        <x:v>高度匹配 AI4Polymer / polymer informatics：期刊明确聚焦化学、材料、生物技术与机器学习/AI、自动化、数据驱动发现的交叉研究。强调方法如何加速科学发现、可复现和数据基础。</x:v>
       </x:c>
       <x:c r="F15" s="25" t="str">
-        <x:v>待核验：需查官网 Aims &amp; Scope</x:v>
+        <x:v>RSC Gold OA 期刊；关注实验和理论研究如何借助机器学习、自动化/机器人、数据库及数据分析加速发现。</x:v>
       </x:c>
       <x:c r="G15" s="25" t="str">
-        <x:v>待核验：需查官网作者指南</x:v>
+        <x:v>Communications、Full Papers、Commit 技术说明、Reviews、Perspectives、Opinions、Comments、Tutorial Reviews。</x:v>
       </x:c>
       <x:c r="H15" s="25" t="str">
-        <x:v>未核验</x:v>
+        <x:v>2024 JIF 5.6（RSC 页面/博客）。RSC 报告接收率 67%，但公开摘要未说明分母和统计窗口，不能当作个人录用概率。</x:v>
       </x:c>
       <x:c r="I15" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>RSC 报告送外审稿件 first decision 平均 45 天；该指标只覆盖被送审稿件。投稿至接收与接收至上线的同口径中位数未核到。</x:v>
       </x:c>
       <x:c r="J15" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>投稿至接收与接收至上线的同口径中位数未核到</x:v>
       </x:c>
       <x:c r="K15" s="25" t="str">
         <x:v>未公开/待核验</x:v>
       </x:c>
       <x:c r="L15" s="25" t="str">
-        <x:v>待核验</x:v>
+        <x:v>Gold OA。自 2026-01-01 投稿适用标准 APC £2,200，另计适用税费；印度、印度尼西亚、菲律宾适用区域价 £1,100；RSC 协议可覆盖，Research4Life A/B 可申请减免，会员/机构折扣条件需核验。</x:v>
       </x:c>
       <x:c r="M15" s="25" t="str">
-        <x:v>未核验</x:v>
+        <x:v>Royal Society of Chemistry</x:v>
       </x:c>
       <x:c r="N15" s="25" t="str">
-        <x:v>待核验</x:v>
+        <x:v>2635-098X (online)</x:v>
       </x:c>
       <x:c r="O15" s="25" t="str">
         <x:v>未公开/未找到可比官方统计</x:v>
@@ -1796,10 +1823,13 @@
         <x:v>待逐刊核验</x:v>
       </x:c>
       <x:c r="W15" s="25" t="str">
-        <x:v>基础目录（逐刊待核验）</x:v>
+        <x:v>官方资料已核验（重点期刊）</x:v>
       </x:c>
       <x:c r="X15" s="25" t="str">
-        <x:v>待核验：期刊官网</x:v>
+        <x:v>https://www.rsc.org/publishing/journals/digital-discovery
+https://www.rsc.org/publishing/publish-with-us/publish-a-journal-article/digital-discovery
+https://pubs.rsc.org/en/journals/journal/dd
+https://blogs.rsc.org/dd</x:v>
       </x:c>
       <x:c r="Y15" s="25" t="str">
         <x:v>所给 WoS 汇总表频次；原检索期和窗口未提供</x:v>
@@ -1819,34 +1849,34 @@
         <x:v>综合/其他</x:v>
       </x:c>
       <x:c r="E16" s="25" t="str">
-        <x:v>根据期刊名称/学科线索的初步分类；需结合官网 aims &amp; scope 和近年相关文章判断。</x:v>
+        <x:v>综合性 OA 期刊，聚合物信息学需体现对相关专业社群有意义的重要科学进展，通常需要扎实机制/实验或跨领域验证；不以单纯应用预测为充分贡献。</x:v>
       </x:c>
       <x:c r="F16" s="25" t="str">
-        <x:v>待核验：需查官网 Aims &amp; Scope</x:v>
+        <x:v>覆盖自然科学各领域，发表对特定专业社群重要的原创研究。Nature Communication 按官方刊名规范为 Nature Communications。</x:v>
       </x:c>
       <x:c r="G16" s="25" t="str">
-        <x:v>待核验：需查官网作者指南</x:v>
+        <x:v>Articles、Registered Reports；Reviews、Perspectives、Comments 多为邀稿，另有 Matters Arising 等栏目。</x:v>
       </x:c>
       <x:c r="H16" s="25" t="str">
-        <x:v>未核验</x:v>
+        <x:v>JIF 18.1；5-year JIF 18.9（2025 Nature Portfolio 指标）。</x:v>
       </x:c>
       <x:c r="I16" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>2025 中位数：投稿至首次编辑决定 9 天；投稿至接收 242 天（包含同行评审和作者返修）。9 天可能包含编辑筛选，外审时长及接收至上线未单独公布。</x:v>
       </x:c>
       <x:c r="J16" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>投稿至接收 242 天（包含同行评审和作者返修）</x:v>
       </x:c>
       <x:c r="K16" s="25" t="str">
         <x:v>未公开/待核验</x:v>
       </x:c>
       <x:c r="L16" s="25" t="str">
-        <x:v>待核验</x:v>
+        <x:v>全 OA，研究论文接收后需支付 APC；无投稿费或版面费。当前 APC 总额本次未能核定，税费和机构协议/减免按官方 OA 页面查询。</x:v>
       </x:c>
       <x:c r="M16" s="25" t="str">
-        <x:v>未核验</x:v>
+        <x:v>Springer Nature</x:v>
       </x:c>
       <x:c r="N16" s="25" t="str">
-        <x:v>待核验</x:v>
+        <x:v>2041-1723 (online)</x:v>
       </x:c>
       <x:c r="O16" s="25" t="str">
         <x:v>未公开/未找到可比官方统计</x:v>
@@ -1873,10 +1903,14 @@
         <x:v>待逐刊核验</x:v>
       </x:c>
       <x:c r="W16" s="25" t="str">
-        <x:v>基础目录（逐刊待核验）</x:v>
+        <x:v>官方资料已核验（重点期刊）</x:v>
       </x:c>
       <x:c r="X16" s="25" t="str">
-        <x:v>待核验：期刊官网</x:v>
+        <x:v>https://www.nature.com/ncomms/journal-information
+https://www.nature.com/ncomms/submit/content-types
+https://www.nature.com/nature-portfolio/about-journals/journal-metrics
+https://www.nature.com/ncomms/submit/how-to-submit
+https://www.nature.com/ncomms/open-access</x:v>
       </x:c>
       <x:c r="Y16" s="25" t="str">
         <x:v>所给 WoS 汇总表频次；原检索期和窗口未提供</x:v>
@@ -2053,31 +2087,31 @@
         <x:v>应用导向的聚合物研究。适合把机器学习/模拟与结构-加工-形貌-化学-性能/功能关系、机制或具体应用相连，并有充分验证的工作。纯数据报告通常不合适。</x:v>
       </x:c>
       <x:c r="F19" s="25" t="str">
-        <x:v>跨工程、化学、物理、生物与应用聚合物；含能量、分离/膜、黏合剂、涂层、传感、电子、光子、生物材料、纳米复合材料。</x:v>
+        <x:v>跨工程、化学、物理、生物与应用聚合物；涉及结构、加工、形貌、化学、性质和功能关系。</x:v>
       </x:c>
       <x:c r="G19" s="25" t="str">
         <x:v>Letters、Articles、Reviews、Spotlights on Applications（邀稿）、Forum Articles（邀稿）、Comments。</x:v>
       </x:c>
       <x:c r="H19" s="25" t="str">
-        <x:v>JIF 5.2；CiteScore 7.1（ACS 页面显示，访问时点需复核年份）。</x:v>
+        <x:v>JIF 5.2；5-year JIF 5.0；CiteScore 7.1（ACS Journal Metrics 页面，2026-06-17 数据快照；指标年份需投稿时核对）。</x:v>
       </x:c>
       <x:c r="I19" s="25" t="str">
-        <x:v>未找到该刊官方公开的投稿到首决/接收中位数</x:v>
+        <x:v>ACS 中位数：投稿至无外审编辑决定 5.4 天；投稿至含同行评审决定 34.8 天；投稿至接收 70.2 天（含作者返修时间）；接收至 ASAP 7.4 天（含校样批准）。</x:v>
       </x:c>
       <x:c r="J19" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>投稿至接收 70.2 天（含作者返修时间）</x:v>
       </x:c>
       <x:c r="K19" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>接收至 ASAP 7.4 天（含校样批准）</x:v>
       </x:c>
       <x:c r="L19" s="25" t="str">
-        <x:v>订阅/混合 OA；APC 依据 ACS 当前价目与协议查询。可能有 read-and-publish 机构覆盖。</x:v>
+        <x:v>订阅/混合 OA；可选 OA，也可走订阅路线。APC 应按 ACS 当前价目、税费和机构 Read-and-Publish 协议核算；本次未核定具体总额。</x:v>
       </x:c>
       <x:c r="M19" s="25" t="str">
         <x:v>American Chemical Society</x:v>
       </x:c>
       <x:c r="N19" s="25" t="str">
-        <x:v>2637-6105 (eISSN)</x:v>
+        <x:v>2637-6105 (online)</x:v>
       </x:c>
       <x:c r="O19" s="25" t="str">
         <x:v>未公开/未找到可比官方统计</x:v>
@@ -2107,7 +2141,7 @@
         <x:v>官方资料已核验（重点期刊）</x:v>
       </x:c>
       <x:c r="X19" s="25" t="str">
-        <x:v>https://pubs.acs.org/acsapm
+        <x:v>https://pubs.acs.org/journal-metrics
 https://researcher-resources.acs.org/publish/author_guidelines?coden=aapmcd
 https://pubs.acs.org/aapmcd/pages/info-for-authors</x:v>
       </x:c>
@@ -5429,7 +5463,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R970b84b9d33a4cf8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9965bbc7d8ac44a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5438,63 +5472,63 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="65" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="44" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="36" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="36" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="50" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="46" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="56" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="56" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="50" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="68" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="54" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="50" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="58" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="56" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="48" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="62" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="52" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="58" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="20" t="str">
+      <x:c r="A1" s="34" t="str">
         <x:v>Journal</x:v>
       </x:c>
-      <x:c r="B1" s="20" t="str">
+      <x:c r="B1" s="34" t="str">
         <x:v>WoS records</x:v>
       </x:c>
-      <x:c r="C1" s="20" t="str">
+      <x:c r="C1" s="34" t="str">
         <x:v>Research fit / scope</x:v>
       </x:c>
-      <x:c r="D1" s="20" t="str">
+      <x:c r="D1" s="34" t="str">
         <x:v>Article types</x:v>
       </x:c>
-      <x:c r="E1" s="20" t="str">
+      <x:c r="E1" s="34" t="str">
         <x:v>Metrics</x:v>
       </x:c>
-      <x:c r="F1" s="20" t="str">
+      <x:c r="F1" s="34" t="str">
         <x:v>First decision</x:v>
       </x:c>
-      <x:c r="G1" s="20" t="str">
+      <x:c r="G1" s="34" t="str">
         <x:v>Submission to acceptance</x:v>
       </x:c>
-      <x:c r="H1" s="20" t="str">
+      <x:c r="H1" s="34" t="str">
         <x:v>Acceptance to online</x:v>
       </x:c>
-      <x:c r="I1" s="20" t="str">
+      <x:c r="I1" s="34" t="str">
         <x:v>OA and fee</x:v>
       </x:c>
-      <x:c r="J1" s="20" t="str">
+      <x:c r="J1" s="34" t="str">
         <x:v>Publisher / ISSN</x:v>
       </x:c>
-      <x:c r="K1" s="20" t="str">
+      <x:c r="K1" s="34" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="L1" s="20" t="str">
+      <x:c r="L1" s="34" t="str">
         <x:v>Time</x:v>
       </x:c>
-      <x:c r="M1" s="20" t="str">
+      <x:c r="M1" s="34" t="str">
         <x:v>Fee</x:v>
       </x:c>
-      <x:c r="N1" s="20" t="str">
+      <x:c r="N1" s="34" t="str">
         <x:v>Source links</x:v>
       </x:c>
     </x:row>
@@ -5518,10 +5552,10 @@
         <x:v>投稿至首个编辑决定：13.4 天</x:v>
       </x:c>
       <x:c r="G2" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
+        <x:v>投稿至首个编辑决定：13.4 天；接收到发表：2.7 天。官网称为 2026 上半年发表论文的中位数；不是首轮外审时长或投稿至接收。</x:v>
       </x:c>
       <x:c r="H2" s="25" t="str">
-        <x:v>Median 2.7 days (2026 H1)</x:v>
+        <x:v>未公开/待核验</x:v>
       </x:c>
       <x:c r="I2" s="25" t="str">
         <x:v>全 OA；APC CHF 2,700，适用税费另计；接受后开票。官网列机构 IOAP 与学会折扣。</x:v>
@@ -5546,147 +5580,469 @@
     </x:row>
     <x:row r="3" ht="82" customHeight="1">
       <x:c r="A3" s="25" t="str">
+        <x:v>ACS APPLIED POLYMER MATERIALS</x:v>
+      </x:c>
+      <x:c r="B3" s="25" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C3" s="25" t="str">
+        <x:v>应用导向的聚合物研究。适合把机器学习/模拟与结构-加工-形貌-化学-性能/功能关系、机制或具体应用相连，并有充分验证的工作。纯数据报告通常不合适。</x:v>
+      </x:c>
+      <x:c r="D3" s="25" t="str">
+        <x:v>Letters、Articles、Reviews、Spotlights on Applications（邀稿）、Forum Articles（邀稿）、Comments。</x:v>
+      </x:c>
+      <x:c r="E3" s="25" t="str">
+        <x:v>JIF 5.2；5-year JIF 5.0；CiteScore 7.1（ACS Journal Metrics 页面，2026-06-17 数据快照；指标年份需投稿时核对）。</x:v>
+      </x:c>
+      <x:c r="F3" s="25" t="str">
+        <x:v>ACS 中位数：投稿至无外审编辑决定 5.4 天</x:v>
+      </x:c>
+      <x:c r="G3" s="25" t="str">
+        <x:v>ACS 中位数：投稿至无外审编辑决定 5.4 天；投稿至含同行评审决定 34.8 天；投稿至接收 70.2 天（含作者返修时间）；接收至 ASAP 7.4 天（含校样批准）。</x:v>
+      </x:c>
+      <x:c r="H3" s="25" t="str">
+        <x:v>接收至 ASAP 7.4 天（含校样批准）。</x:v>
+      </x:c>
+      <x:c r="I3" s="25" t="str">
+        <x:v>订阅/混合 OA；可选 OA，也可走订阅路线。APC 应按 ACS 当前价目、税费和机构 Read-and-Publish 协议核算；本次未核定具体总额。</x:v>
+      </x:c>
+      <x:c r="J3" s="25" t="str">
+        <x:v>American Chemical Society / 2637-6105 (online)</x:v>
+      </x:c>
+      <x:c r="K3" s="25" t="str">
+        <x:v>跨工程、化学、物理、生物与应用聚合物；涉及结构、加工、形貌、化学、性质和功能关系。</x:v>
+      </x:c>
+      <x:c r="L3" s="25" t="str">
+        <x:v>ACS 中位数：投稿至无外审编辑决定 5.4 天；投稿至含同行评审决定 34.8 天；投稿至接收 70.2 天（含作者返修时间）；接收至 ASAP 7.4 天（含校样批准）。</x:v>
+      </x:c>
+      <x:c r="M3" s="25" t="str">
+        <x:v>订阅/混合 OA；可选 OA，也可走订阅路线。APC 应按 ACS 当前价目、税费和机构 Read-and-Publish 协议核算；本次未核定具体总额。</x:v>
+      </x:c>
+      <x:c r="N3" s="25" t="str">
+        <x:v>ACS 指标和分阶段时长: https://pubs.acs.org/journal-metrics
+作者指南/范围/稿型: https://researcher-resources.acs.org/publish/author_guidelines?coden=aapmcd
+作者信息/OA: https://pubs.acs.org/aapmcd/pages/info-for-authors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="82" customHeight="1">
+      <x:c r="A4" s="25" t="str">
         <x:v>JOURNAL OF CHEMICAL INFORMATION AND MODELING</x:v>
       </x:c>
-      <x:c r="B3" s="25" t="n">
+      <x:c r="B4" s="25" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="C3" s="25" t="str">
+      <x:c r="C4" s="25" t="str">
         <x:v>计算化学、化学信息学、分子建模与机器学习方法强相关。聚合物稿件要清楚解释方法对化学/材料问题的普适贡献、数据可靠性和外部验证。</x:v>
       </x:c>
-      <x:c r="D3" s="25" t="str">
+      <x:c r="D4" s="25" t="str">
         <x:v>期刊作者指南列有原创研究等类型；按最新 ACS author guidelines 核对。</x:v>
       </x:c>
-      <x:c r="E3" s="25" t="str">
+      <x:c r="E4" s="25" t="str">
         <x:v>JIF 6.4、5 年 IF 6.9、CiteScore 8.8（ACS 页面，数据 as of 2025）。</x:v>
       </x:c>
-      <x:c r="F3" s="25" t="str">
+      <x:c r="F4" s="25" t="str">
         <x:v>首个同行评审决定中位数 31.3 天</x:v>
       </x:c>
-      <x:c r="G3" s="25" t="str">
-        <x:v>Median 76.3 days (2025)</x:v>
-      </x:c>
-      <x:c r="H3" s="25" t="str">
-        <x:v>Median 9.6 days (2025)</x:v>
-      </x:c>
-      <x:c r="I3" s="25" t="str">
+      <x:c r="G4" s="25" t="str">
+        <x:v>首个同行评审决定中位数 31.3 天；投稿到接收 76.3 天；接收至 ASAP 9.6 天（ACS 页面，2025；口径并非每个处理阶段）。</x:v>
+      </x:c>
+      <x:c r="H4" s="25" t="str">
+        <x:v>接收至 ASAP 9.6 天（ACS 页面，2025</x:v>
+      </x:c>
+      <x:c r="I4" s="25" t="str">
         <x:v>混合 OA，可选 CC BY/CC BY-NC-ND；非 OA 订阅路线可用。费用按 ACS 最新价目/协议核实。</x:v>
       </x:c>
-      <x:c r="J3" s="25" t="str">
+      <x:c r="J4" s="25" t="str">
         <x:v>American Chemical Society / 1549-9596 (eISSN)</x:v>
       </x:c>
-      <x:c r="K3" s="25" t="str">
+      <x:c r="K4" s="25" t="str">
         <x:v>化学信息学与分子建模：AI/ML、分子模拟、多尺度建模、软件算法、化学数据分析等。</x:v>
       </x:c>
-      <x:c r="L3" s="25" t="str">
+      <x:c r="L4" s="25" t="str">
         <x:v>首个同行评审决定中位数 31.3 天；投稿到接收 76.3 天；接收至 ASAP 9.6 天（ACS 页面，2025；口径并非每个处理阶段）。</x:v>
       </x:c>
-      <x:c r="M3" s="25" t="str">
+      <x:c r="M4" s="25" t="str">
         <x:v>混合 OA，可选 CC BY/CC BY-NC-ND；非 OA 订阅路线可用。费用按 ACS 最新价目/协议核实。</x:v>
       </x:c>
-      <x:c r="N3" s="25" t="str">
+      <x:c r="N4" s="25" t="str">
         <x:v>期刊范围/指标: https://pubs.acs.org/page/jcisd8/about.html
 作者信息: https://pubs.acs.org/jcisd8/pages/info-for-authors
 ACS 指标: https://pubs.acs.org/journal-metrics</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="82" customHeight="1">
-      <x:c r="A4" s="25" t="str">
+    <x:row r="5" ht="82" customHeight="1">
+      <x:c r="A5" s="25" t="str">
         <x:v>NPJ COMPUTATIONAL MATERIALS</x:v>
       </x:c>
-      <x:c r="B4" s="25" t="n">
+      <x:c r="B5" s="25" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="C4" s="25" t="str">
+      <x:c r="C5" s="25" t="str">
         <x:v>面向计算材料科学方法及其重要应用。适合有显著方法学或材料学进展、可信验证且聚合物问题有广泛意义的工作；通常要求高影响和清楚的计算贡献。</x:v>
       </x:c>
-      <x:c r="D4" s="25" t="str">
+      <x:c r="D5" s="25" t="str">
         <x:v>Research Articles、Reviews &amp; Analysis、News &amp; Comment 等；核对内容类型指南。</x:v>
       </x:c>
-      <x:c r="E4" s="25" t="str">
+      <x:c r="E5" s="25" t="str">
         <x:v>JIF 13.1、5 年 JIF 13.7、SJR 2.943（2025）。</x:v>
       </x:c>
-      <x:c r="F4" s="25" t="str">
+      <x:c r="F5" s="25" t="str">
         <x:v>投稿至首个编辑决定中位数 14 天</x:v>
       </x:c>
-      <x:c r="G4" s="25" t="str">
-        <x:v>Median 136 days (2025)</x:v>
-      </x:c>
-      <x:c r="H4" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
-      </x:c>
-      <x:c r="I4" s="25" t="str">
+      <x:c r="G5" s="25" t="str">
+        <x:v>投稿至首个编辑决定中位数 14 天；投稿至接收中位数 136 天（Springer Nature 官方，2025）。首决可能含编辑筛选。</x:v>
+      </x:c>
+      <x:c r="H5" s="25" t="str">
+        <x:v>未公开/待核验</x:v>
+      </x:c>
+      <x:c r="I5" s="25" t="str">
         <x:v>全 OA；原创研究 APC £2,790 / $3,590 / €3,090；税费可能另计；机构协议与低收入国家减免可查询。</x:v>
       </x:c>
-      <x:c r="J4" s="25" t="str">
+      <x:c r="J5" s="25" t="str">
         <x:v>Springer Nature 与中国科学院上海硅酸盐研究所合作出版 / 2057-3960 (online)</x:v>
       </x:c>
-      <x:c r="K4" s="25" t="str">
+      <x:c r="K5" s="25" t="str">
         <x:v>开发与应用计算材料科学技术，跨材料体系。</x:v>
       </x:c>
-      <x:c r="L4" s="25" t="str">
+      <x:c r="L5" s="25" t="str">
         <x:v>投稿至首个编辑决定中位数 14 天；投稿至接收中位数 136 天（Springer Nature 官方，2025）。首决可能含编辑筛选。</x:v>
       </x:c>
-      <x:c r="M4" s="25" t="str">
+      <x:c r="M5" s="25" t="str">
         <x:v>全 OA；原创研究 APC £2,790 / $3,590 / €3,090；税费可能另计；机构协议与低收入国家减免可查询。</x:v>
       </x:c>
-      <x:c r="N4" s="25" t="str">
+      <x:c r="N5" s="25" t="str">
         <x:v>期刊信息/索引: https://www.nature.com/npjcompumats/for-authors-and-referees/guide-to-authors/about/journal-information
 指标与时间: https://www.nature.com/npjcompumats/journal-impact
 OA/APC: https://www.nature.com/npjcompumats/for-authors-and-referees/guide-to-authors/about/open-access
 范围: https://www.nature.com/npjcompumats/aims-and-scope</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="82" customHeight="1">
-      <x:c r="A5" s="25" t="str">
-        <x:v>ACS APPLIED POLYMER MATERIALS</x:v>
-      </x:c>
-      <x:c r="B5" s="25" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C5" s="25" t="str">
-        <x:v>应用导向的聚合物研究。适合把机器学习/模拟与结构-加工-形貌-化学-性能/功能关系、机制或具体应用相连，并有充分验证的工作。纯数据报告通常不合适。</x:v>
-      </x:c>
-      <x:c r="D5" s="25" t="str">
-        <x:v>Letters、Articles、Reviews、Spotlights on Applications（邀稿）、Forum Articles（邀稿）、Comments。</x:v>
-      </x:c>
-      <x:c r="E5" s="25" t="str">
-        <x:v>JIF 5.2；CiteScore 7.1（ACS 页面显示，访问时点需复核年份）。</x:v>
-      </x:c>
-      <x:c r="F5" s="25" t="str">
-        <x:v>未找到该刊官方公开的投稿到首决/接收中位数</x:v>
-      </x:c>
-      <x:c r="G5" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
-      </x:c>
-      <x:c r="H5" s="25" t="str">
-        <x:v>未公开/待核验</x:v>
-      </x:c>
-      <x:c r="I5" s="25" t="str">
-        <x:v>订阅/混合 OA；APC 依据 ACS 当前价目与协议查询。可能有 read-and-publish 机构覆盖。</x:v>
-      </x:c>
-      <x:c r="J5" s="25" t="str">
-        <x:v>American Chemical Society / 2637-6105 (eISSN)</x:v>
-      </x:c>
-      <x:c r="K5" s="25" t="str">
-        <x:v>跨工程、化学、物理、生物与应用聚合物；含能量、分离/膜、黏合剂、涂层、传感、电子、光子、生物材料、纳米复合材料。</x:v>
-      </x:c>
-      <x:c r="L5" s="25" t="str">
-        <x:v>未找到该刊官方公开的投稿到首决/接收中位数；需看作者样本。</x:v>
-      </x:c>
-      <x:c r="M5" s="25" t="str">
-        <x:v>订阅/混合 OA；APC 依据 ACS 当前价目与协议查询。可能有 read-and-publish 机构覆盖。</x:v>
-      </x:c>
-      <x:c r="N5" s="25" t="str">
-        <x:v>期刊主页与指标: https://pubs.acs.org/acsapm
-作者指南/范围/稿件类型: https://researcher-resources.acs.org/publish/author_guidelines?coden=aapmcd
-作者信息/OA: https://pubs.acs.org/aapmcd/pages/info-for-authors</x:v>
+    <x:row r="6">
+      <x:c r="A6" s="25" t="str">
+        <x:v>MACROMOLECULES</x:v>
+      </x:c>
+      <x:c r="B6" s="25" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="C6" s="25" t="str">
+        <x:v>基础聚合物科学定位强，涵盖合成、结构、物理化学、表征、加工及理论/模拟。聚合物信息学投稿应提出对高分子科学有解释力的发现，不宜只展示模型分数。</x:v>
+      </x:c>
+      <x:c r="D6" s="25" t="str">
+        <x:v>Articles；期刊也刊发综述、观点/专题等类型，当前投稿分类与邀请要求以 ACS 作者指南为准。</x:v>
+      </x:c>
+      <x:c r="E6" s="25" t="str">
+        <x:v>JIF 5.7；5-year JIF 5.5；CiteScore 8.8（ACS Journal Metrics 页面，2026-06-17 数据快照；指标年份仍应按投稿时核对）。</x:v>
+      </x:c>
+      <x:c r="F6" s="25" t="str">
+        <x:v>ACS 中位数：投稿至无外审编辑决定 3.9 天</x:v>
+      </x:c>
+      <x:c r="G6" s="25" t="str">
+        <x:v>ACS 中位数：投稿至无外审编辑决定 3.9 天；投稿至含同行评审决定 34 天；投稿至接收 86 天（含作者返修时间）；接收至 ASAP 8.4 天（含校样批准）。这些阶段不是单纯外审用时。</x:v>
+      </x:c>
+      <x:c r="H6" s="25" t="str">
+        <x:v>接收至 ASAP 8.4 天（含校样批准）。</x:v>
+      </x:c>
+      <x:c r="I6" s="25" t="str">
+        <x:v>混合/可选 OA；可走订阅发表。OA APC 金额随 ACS 价目、币种、税费与机构协议变化，本次未核定应付总额。</x:v>
+      </x:c>
+      <x:c r="J6" s="25" t="str">
+        <x:v>American Chemical Society / 0024-9297 (print); 1520-5835 (online)</x:v>
+      </x:c>
+      <x:c r="K6" s="25" t="str">
+        <x:v>ACS 将其定位为发表前沿聚合物科学研究的同行评审期刊；理论、实验、模拟与跨学科工作均可考虑。</x:v>
+      </x:c>
+      <x:c r="L6" s="25" t="str">
+        <x:v>ACS 中位数：投稿至无外审编辑决定 3.9 天；投稿至含同行评审决定 34 天；投稿至接收 86 天（含作者返修时间）；接收至 ASAP 8.4 天（含校样批准）。这些阶段不是单纯外审用时。</x:v>
+      </x:c>
+      <x:c r="M6" s="25" t="str">
+        <x:v>混合/可选 OA；可走订阅发表。OA APC 金额随 ACS 价目、币种、税费与机构协议变化，本次未核定应付总额。</x:v>
+      </x:c>
+      <x:c r="N6" s="25" t="str">
+        <x:v>期刊主页/范围: https://pubs.acs.org/journal/macromolecules
+ACS 指标和分阶段时长: https://pubs.acs.org/journal-metrics
+作者指南: https://pubs.acs.org/mamobx/pages/info-for-authors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="25" t="str">
+        <x:v>CHEMICAL ENGINEERING JOURNAL</x:v>
+      </x:c>
+      <x:c r="B7" s="25" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="C7" s="25" t="str">
+        <x:v>适合将聚合物信息学与化工过程、反应/分离、能源/环境技术、规模化加工或可量化工程性能联系起来的研究。仅有材料性质预测、缺少化工问题或验证时匹配度较低。</x:v>
+      </x:c>
+      <x:c r="D7" s="25" t="str">
+        <x:v>Research Articles、Review Articles、Short Communications 等；具体栏目和字数按最新版 Elsevier Guide for Authors 核验。</x:v>
+      </x:c>
+      <x:c r="E7" s="25" t="str">
+        <x:v>ScienceDirect 期刊页显示 Impact Factor 12.5、CiteScore 19.6（页面动态指标快照；年份口径应投稿前复核）。</x:v>
+      </x:c>
+      <x:c r="F7" s="25" t="str">
+        <x:v>官方公开页面未核到可比的投稿至首决、送外审首决、投稿至接收或接收到在线发表中位数</x:v>
+      </x:c>
+      <x:c r="G7" s="25" t="str">
+        <x:v>官方公开页面未核到可比的投稿至首决、送外审首决、投稿至接收或接收到在线发表中位数；分别标记未公开。</x:v>
+      </x:c>
+      <x:c r="H7" s="25" t="str">
+        <x:v>未公开/待核验</x:v>
+      </x:c>
+      <x:c r="I7" s="25" t="str">
+        <x:v>ScienceDirect 标注支持 OA；为订阅/混合路线的选择情况及最新 APC、税费和机构协议，本次未确认具体金额，投稿时查看官方 OA 成本计算器。</x:v>
+      </x:c>
+      <x:c r="J7" s="25" t="str">
+        <x:v>Elsevier / 1385-8947 (print); 1873-3212 (online)</x:v>
+      </x:c>
+      <x:c r="K7" s="25" t="str">
+        <x:v>工程应用驱动的化学工程研究；聚合物工作需清晰体现过程、系统或应用层面的化工价值。</x:v>
+      </x:c>
+      <x:c r="L7" s="25" t="str">
+        <x:v>官方公开页面未核到可比的投稿至首决、送外审首决、投稿至接收或接收到在线发表中位数；分别标记未公开。</x:v>
+      </x:c>
+      <x:c r="M7" s="25" t="str">
+        <x:v>ScienceDirect 标注支持 OA；为订阅/混合路线的选择情况及最新 APC、税费和机构协议，本次未确认具体金额，投稿时查看官方 OA 成本计算器。</x:v>
+      </x:c>
+      <x:c r="N7" s="25" t="str">
+        <x:v>ScienceDirect 期刊主页/指标: https://www.sciencedirect.com/journal/chemical-engineering-journal
+作者指南: https://www.sciencedirect.com/journal/chemical-engineering-journal/publish/guide-for-authors
+官方期刊页面快照: https://www.sciencedirect.com/journal/chemical-engineering-journal/vol/226/suppl/C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="25" t="str">
+        <x:v>POLYMER</x:v>
+      </x:c>
+      <x:c r="B8" s="25" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="C8" s="25" t="str">
+        <x:v>传统聚合物科学与技术综合刊。匹配合成、结构/性能、物理化学、表征、加工、应用，以及具有明确高分子科学贡献的建模与机器学习研究。</x:v>
+      </x:c>
+      <x:c r="D8" s="25" t="str">
+        <x:v>Research/Regular Articles、Review Articles、Short Communications（以当前作者指南为准）。</x:v>
+      </x:c>
+      <x:c r="E8" s="25" t="str">
+        <x:v>ScienceDirect 官方期刊页面快照显示 Impact Factor 4.5、CiteScore 7.4；该快照指标年份未明确，不能作为当前年份保证值。</x:v>
+      </x:c>
+      <x:c r="F8" s="25" t="str">
+        <x:v>未核到官网公布的首个编辑决定、外审首决、投稿至接收和接收至在线发表中位数。</x:v>
+      </x:c>
+      <x:c r="G8" s="25" t="str">
+        <x:v>未核到官网公布的首个编辑决定、外审首决、投稿至接收和接收至在线发表中位数。</x:v>
+      </x:c>
+      <x:c r="H8" s="25" t="str">
+        <x:v>接收至在线发表中位数。</x:v>
+      </x:c>
+      <x:c r="I8" s="25" t="str">
+        <x:v>ScienceDirect 标注支持 Open Access；按订阅/混合期刊路线处理。当前 APC、税费、协议覆盖需从官方作者端重新确认。</x:v>
+      </x:c>
+      <x:c r="J8" s="25" t="str">
+        <x:v>Elsevier / 0032-3861 (print); 1873-2291 (online)</x:v>
+      </x:c>
+      <x:c r="K8" s="25" t="str">
+        <x:v>覆盖聚合物科学和技术；计算研究应给出与聚合物现象、机制或应用相关的可验证贡献。</x:v>
+      </x:c>
+      <x:c r="L8" s="25" t="str">
+        <x:v>未核到官网公布的首个编辑决定、外审首决、投稿至接收和接收至在线发表中位数。</x:v>
+      </x:c>
+      <x:c r="M8" s="25" t="str">
+        <x:v>ScienceDirect 标注支持 Open Access；按订阅/混合期刊路线处理。当前 APC、税费、协议覆盖需从官方作者端重新确认。</x:v>
+      </x:c>
+      <x:c r="N8" s="25" t="str">
+        <x:v>ScienceDirect 期刊主页: https://www.sciencedirect.com/journal/polymer
+作者指南: https://www.sciencedirect.com/journal/polymer/publish/guide-for-authors
+官方期刊页面快照/指标与稿型: https://www.sciencedirect.com/journal/polymer/vol/298/suppl/C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="25" t="str">
+        <x:v>DIGITAL DISCOVERY</x:v>
+      </x:c>
+      <x:c r="B9" s="25" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C9" s="25" t="str">
+        <x:v>高度匹配 AI4Polymer / polymer informatics：期刊明确聚焦化学、材料、生物技术与机器学习/AI、自动化、数据驱动发现的交叉研究。强调方法如何加速科学发现、可复现和数据基础。</x:v>
+      </x:c>
+      <x:c r="D9" s="25" t="str">
+        <x:v>Communications、Full Papers、Commit 技术说明、Reviews、Perspectives、Opinions、Comments、Tutorial Reviews。</x:v>
+      </x:c>
+      <x:c r="E9" s="25" t="str">
+        <x:v>2024 JIF 5.6（RSC 页面/博客）。RSC 报告接收率 67%，但公开摘要未说明分母和统计窗口，不能当作个人录用概率。</x:v>
+      </x:c>
+      <x:c r="F9" s="25" t="str">
+        <x:v>RSC 报告送外审稿件 first decision 平均 45 天</x:v>
+      </x:c>
+      <x:c r="G9" s="25" t="str">
+        <x:v>RSC 报告送外审稿件 first decision 平均 45 天；该指标只覆盖被送审稿件。投稿至接收与接收至上线的同口径中位数未核到。</x:v>
+      </x:c>
+      <x:c r="H9" s="25" t="str">
+        <x:v>未公开/待核验</x:v>
+      </x:c>
+      <x:c r="I9" s="25" t="str">
+        <x:v>Gold OA。自 2026-01-01 投稿适用标准 APC £2,200，另计适用税费；印度、印度尼西亚、菲律宾适用区域价 £1,100；RSC 协议可覆盖，Research4Life A/B 可申请减免，会员/机构折扣条件需核验。</x:v>
+      </x:c>
+      <x:c r="J9" s="25" t="str">
+        <x:v>Royal Society of Chemistry / 2635-098X (online)</x:v>
+      </x:c>
+      <x:c r="K9" s="25" t="str">
+        <x:v>RSC Gold OA 期刊；关注实验和理论研究如何借助机器学习、自动化/机器人、数据库及数据分析加速发现。</x:v>
+      </x:c>
+      <x:c r="L9" s="25" t="str">
+        <x:v>RSC 报告送外审稿件 first decision 平均 45 天；该指标只覆盖被送审稿件。投稿至接收与接收至上线的同口径中位数未核到。</x:v>
+      </x:c>
+      <x:c r="M9" s="25" t="str">
+        <x:v>Gold OA。自 2026-01-01 投稿适用标准 APC £2,200，另计适用税费；印度、印度尼西亚、菲律宾适用区域价 £1,100；RSC 协议可覆盖，Research4Life A/B 可申请减免，会员/机构折扣条件需核验。</x:v>
+      </x:c>
+      <x:c r="N9" s="25" t="str">
+        <x:v>RSC 期刊范围/稿型: https://www.rsc.org/publishing/journals/digital-discovery
+投稿指南/APC/减免: https://www.rsc.org/publishing/publish-with-us/publish-a-journal-article/digital-discovery
+RSC 期刊信息/审稿统计: https://pubs.rsc.org/en/journals/journal/dd
+RSC 期刊博客/指标与接收率: https://blogs.rsc.org/dd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="25" t="str">
+        <x:v>NATURE COMMUNICATIONS</x:v>
+      </x:c>
+      <x:c r="B10" s="25" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C10" s="25" t="str">
+        <x:v>综合性 OA 期刊，聚合物信息学需体现对相关专业社群有意义的重要科学进展，通常需要扎实机制/实验或跨领域验证；不以单纯应用预测为充分贡献。</x:v>
+      </x:c>
+      <x:c r="D10" s="25" t="str">
+        <x:v>Articles、Registered Reports；Reviews、Perspectives、Comments 多为邀稿，另有 Matters Arising 等栏目。</x:v>
+      </x:c>
+      <x:c r="E10" s="25" t="str">
+        <x:v>JIF 18.1；5-year JIF 18.9（2025 Nature Portfolio 指标）。</x:v>
+      </x:c>
+      <x:c r="F10" s="25" t="str">
+        <x:v>2025 中位数：投稿至首次编辑决定 9 天</x:v>
+      </x:c>
+      <x:c r="G10" s="25" t="str">
+        <x:v>2025 中位数：投稿至首次编辑决定 9 天；投稿至接收 242 天（包含同行评审和作者返修）。9 天可能包含编辑筛选，外审时长及接收至上线未单独公布。</x:v>
+      </x:c>
+      <x:c r="H10" s="25" t="str">
+        <x:v>未公开/待核验</x:v>
+      </x:c>
+      <x:c r="I10" s="25" t="str">
+        <x:v>全 OA，研究论文接收后需支付 APC；无投稿费或版面费。当前 APC 总额本次未能核定，税费和机构协议/减免按官方 OA 页面查询。</x:v>
+      </x:c>
+      <x:c r="J10" s="25" t="str">
+        <x:v>Springer Nature / 2041-1723 (online)</x:v>
+      </x:c>
+      <x:c r="K10" s="25" t="str">
+        <x:v>覆盖自然科学各领域，发表对特定专业社群重要的原创研究。Nature Communication 按官方刊名规范为 Nature Communications。</x:v>
+      </x:c>
+      <x:c r="L10" s="25" t="str">
+        <x:v>2025 中位数：投稿至首次编辑决定 9 天；投稿至接收 242 天（包含同行评审和作者返修）。9 天可能包含编辑筛选，外审时长及接收至上线未单独公布。</x:v>
+      </x:c>
+      <x:c r="M10" s="25" t="str">
+        <x:v>全 OA，研究论文接收后需支付 APC；无投稿费或版面费。当前 APC 总额本次未能核定，税费和机构协议/减免按官方 OA 页面查询。</x:v>
+      </x:c>
+      <x:c r="N10" s="25" t="str">
+        <x:v>期刊信息/范围: https://www.nature.com/ncomms/journal-information
+稿件类型: https://www.nature.com/ncomms/submit/content-types
+2025 指标/同行评审时间: https://www.nature.com/nature-portfolio/about-journals/journal-metrics
+投稿与作者指南: https://www.nature.com/ncomms/submit/how-to-submit
+OA 政策/APC: https://www.nature.com/ncomms/open-access</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="25" t="str">
+        <x:v>NATURE COMPUTATIONAL SCIENCE</x:v>
+      </x:c>
+      <x:c r="B11" s="25"/>
+      <x:c r="C11" s="25" t="str">
+        <x:v>面向跨学科计算科学。聚合物信息学稿件若以新计算方法、数学模型或具有可迁移性的科学发现为核心，并在科学问题上充分验证，匹配度较高；只应用常见模型做单一聚合物数据预测的竞争力可能较弱。</x:v>
+      </x:c>
+      <x:c r="D11" s="25" t="str">
+        <x:v>Articles、Reviews、Perspectives、Brief Communications、Resources、Comments、News &amp; Views 等。</x:v>
+      </x:c>
+      <x:c r="E11" s="25" t="str">
+        <x:v>JIF 20.3；5-year JIF 21.9（2025 Nature Portfolio 指标）。</x:v>
+      </x:c>
+      <x:c r="F11" s="25" t="str">
+        <x:v>2025 中位数：投稿至首次编辑决定 13 天</x:v>
+      </x:c>
+      <x:c r="G11" s="25" t="str">
+        <x:v>2025 中位数：投稿至首次编辑决定 13 天；投稿至接收 193 天。首决可能含编辑筛选；接收至上线和返修轮次未给出同口径中位数。</x:v>
+      </x:c>
+      <x:c r="H11" s="25" t="str">
+        <x:v>未公开/待核验</x:v>
+      </x:c>
+      <x:c r="I11" s="25" t="str">
+        <x:v>混合期刊：可选 Gold OA，也有订阅发表路线。Gold OA APC £9,390 / $12,850 / €10,850（税费与机构协议/减免按页面核验）；非原创研究稿件的 OA 资格有限。</x:v>
+      </x:c>
+      <x:c r="J11" s="25" t="str">
+        <x:v>Springer Nature / 2662-8457 (online)</x:v>
+      </x:c>
+      <x:c r="K11" s="25" t="str">
+        <x:v>发表计算技术、数学模型及其在不同科学领域的应用；采用在线出版和专职编辑团队。</x:v>
+      </x:c>
+      <x:c r="L11" s="25" t="str">
+        <x:v>2025 中位数：投稿至首次编辑决定 13 天；投稿至接收 193 天。首决可能含编辑筛选；接收至上线和返修轮次未给出同口径中位数。</x:v>
+      </x:c>
+      <x:c r="M11" s="25" t="str">
+        <x:v>混合期刊：可选 Gold OA，也有订阅发表路线。Gold OA APC £9,390 / $12,850 / €10,850（税费与机构协议/减免按页面核验）；非原创研究稿件的 OA 资格有限。</x:v>
+      </x:c>
+      <x:c r="N11" s="25" t="str">
+        <x:v>期刊信息/范围/内容类型: https://www.nature.com/natcomputsci/journal-information
+2025 指标与审稿时间: https://www.nature.com/nature-portfolio/about-journals/journal-metrics
+OA 选项/APC: https://www.nature.com/natcomputsci/submission-guidelines/publishing-options</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="25" t="str">
+        <x:v>NATURE MACHINE INTELLIGENCE</x:v>
+      </x:c>
+      <x:c r="B12" s="25"/>
+      <x:c r="C12" s="25" t="str">
+        <x:v>适合提出对 AI/ML 方法或其科学应用有广泛价值、超越单一聚合物体系的研究。仅用常规算法提升某个聚合物数据集指标，通常不足以支撑其广泛方法学/科学意义定位。</x:v>
+      </x:c>
+      <x:c r="D12" s="25" t="str">
+        <x:v>Articles、Analysis、Correspondence、Reviews、Perspectives、Comments、Matters Arising、Reusability Reports 等；部分类型邀稿。</x:v>
+      </x:c>
+      <x:c r="E12" s="25" t="str">
+        <x:v>JIF 29.8；5-year JIF 36.0（2025 Nature Portfolio 指标）。</x:v>
+      </x:c>
+      <x:c r="F12" s="25" t="str">
+        <x:v>2025 中位数：投稿至首次编辑决定 10 天</x:v>
+      </x:c>
+      <x:c r="G12" s="25" t="str">
+        <x:v>2025 中位数：投稿至首次编辑决定 10 天；投稿至接收 231 天。首决主要对应是否送外审，不等于首轮外审；接收后上线未单列。</x:v>
+      </x:c>
+      <x:c r="H12" s="25" t="str">
+        <x:v>未公开/待核验</x:v>
+      </x:c>
+      <x:c r="I12" s="25" t="str">
+        <x:v>混合期刊：可选 Gold OA，也可订阅发表。Gold OA APC £9,390 / $12,850 / €10,850（税费与协议覆盖按官方页面核实）；非原创研究稿件一般不适用 Gold OA。</x:v>
+      </x:c>
+      <x:c r="J12" s="25" t="str">
+        <x:v>Springer Nature / 2522-5839 (online)</x:v>
+      </x:c>
+      <x:c r="K12" s="25" t="str">
+        <x:v>覆盖人工智能和机器学习的开发及其跨学科应用。编辑按研究推进程度、证据/分析可靠性及对广泛读者的相关性决定是否外审。</x:v>
+      </x:c>
+      <x:c r="L12" s="25" t="str">
+        <x:v>2025 中位数：投稿至首次编辑决定 10 天；投稿至接收 231 天。首决主要对应是否送外审，不等于首轮外审；接收后上线未单列。</x:v>
+      </x:c>
+      <x:c r="M12" s="25" t="str">
+        <x:v>混合期刊：可选 Gold OA，也可订阅发表。Gold OA APC £9,390 / $12,850 / €10,850（税费与协议覆盖按官方页面核实）；非原创研究稿件一般不适用 Gold OA。</x:v>
+      </x:c>
+      <x:c r="N12" s="25" t="str">
+        <x:v>期刊范围与内容类型: https://www.nature.com/natmachintell/content
+编辑流程/转投政策: https://www.nature.com/natmachintell/submission-guidelines/editorial-process
+2025 指标与审稿时间: https://www.nature.com/nature-portfolio/about-journals/journal-metrics
+OA 选项/APC: https://www.nature.com/natmachintell/submission-guidelines/publishing-options</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb11958e888ff4569"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2883552ae4c4958"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5776,7 +6132,7 @@
         <x:v>Journal profiles</x:v>
       </x:c>
       <x:c r="B10" s="25" t="str">
-        <x:v>POLYMERS; ACS APPLIED POLYMER MATERIALS; JOURNAL OF CHEMICAL INFORMATION AND MODELING; NPJ COMPUTATIONAL MATERIALS</x:v>
+        <x:v>POLYMERS; ACS APPLIED POLYMER MATERIALS; JOURNAL OF CHEMICAL INFORMATION AND MODELING; NPJ COMPUTATIONAL MATERIALS; MACROMOLECULES; CHEMICAL ENGINEERING JOURNAL; POLYMER; DIGITAL DISCOVERY; NATURE COMMUNICATIONS; NATURE COMPUTATIONAL SCIENCE; NATURE MACHINE INTELLIGENCE</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">
@@ -5828,6 +6184,14 @@
         <x:v>Revisit official scope, APC, metrics and time pages on the date of submission; APCs and agreements can change.</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>Supplementary profiles</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Nature Computational Science and Nature Machine Intelligence were additionally reviewed but do not occur in the supplied 61-title WoS list. They have no WoS record count and are excluded from the dashboard threshold and corpus charts.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>